<commit_message>
scan: seg4 2026-10-13 03:00 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq5_2026-10-12.xlsx
+++ b/output/full_scan/batch_seq5_2026-10-12.xlsx
@@ -2912,21 +2912,21 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>4770</v>
+        <v>6127</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>上品</t>
+          <t>九豪</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>687.9847747280993</v>
+        <v>689.2275388421415</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>270</v>
+        <v>64</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,13 +2937,13 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>57.54230546453094</v>
+        <v>74.00011366866468</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>41.65767001643372</v>
+        <v>26.38051126431226</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.6435542341763623</v>
+        <v>4.677731675619241</v>
       </c>
       <c r="K47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.403898465031828</v>
+        <v>1.62577722689811</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>4912</v>
+        <v>4770</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>聯德控股-KY</t>
+          <t>上品</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>686.2898374884181</v>
+        <v>687.9847747280993</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>106.5</v>
+        <v>270</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,16 +2990,16 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>62.33325002781681</v>
+        <v>57.54230546453094</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>26.59414959522693</v>
+        <v>41.65767001643372</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.9101774346030695</v>
+        <v>0.6435542341763623</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>0</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.9103246934854984</v>
+        <v>-0.403898465031828</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3018,21 +3018,21 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6150</v>
+        <v>4912</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>撼訊</t>
+          <t>聯德控股-KY</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>681.5762585079516</v>
+        <v>686.2898374884181</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>69</v>
+        <v>106.5</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>64.61338062114235</v>
+        <v>62.33325002781681</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>31.90096670840835</v>
+        <v>26.59414959522693</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>1.594223190088411</v>
+        <v>0.9101774346030695</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.3705718625290128</v>
+        <v>0.9103246934854984</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, dealer_buy_3d, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>4571</v>
+        <v>6150</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>鈞興-KY</t>
+          <t>撼訊</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>677.1052617279503</v>
+        <v>681.5762585079516</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>155</v>
+        <v>69</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,16 +3096,16 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>52.40774178283002</v>
+        <v>64.61338062114235</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>10.68540079343118</v>
+        <v>31.90096670840835</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>1.812151140780488</v>
+        <v>1.594223190088411</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.5751390145729502</v>
+        <v>0.3705718625290128</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>volume_break, breakout_20d, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong</t>
+          <t>volume_break, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, dealer_buy_3d, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>4916</v>
+        <v>4571</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>事欣科</t>
+          <t>鈞興-KY</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>668.7505315865416</v>
+        <v>677.1052617279503</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>103</v>
+        <v>155</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,16 +3149,16 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>52.94680697601884</v>
+        <v>52.40774178283002</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>22.2692358242464</v>
+        <v>10.68540079343118</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.4386793854481485</v>
+        <v>1.812151140780488</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.1012395858336594</v>
+        <v>0.5751390145729502</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>volume_break, breakout_20d, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>5347</v>
+        <v>4916</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>世界</t>
+          <t>事欣科</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>667.2654681521942</v>
+        <v>668.7505315865416</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>181</v>
+        <v>103</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,49 +3202,49 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>58.30853505399338</v>
+        <v>52.94680697601884</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>34.67137464159429</v>
+        <v>22.2692358242464</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.7708106069735521</v>
+        <v>0.4386793854481485</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.833155444704758</v>
+        <v>0.1012395858336594</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>5483</v>
+        <v>5347</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>中美晶</t>
+          <t>世界</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>663.7168291409964</v>
+        <v>667.2654681521942</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>213.5</v>
+        <v>181</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,49 +3255,49 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>60.55907416121683</v>
+        <v>58.30853505399338</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>31.10196452451822</v>
+        <v>34.67137464159429</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.3106851250175323</v>
+        <v>0.7708106069735521</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L53" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M53" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>2.478466658357904</v>
+        <v>0.833155444704758</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, invest_trust_buy_2d, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>4960</v>
+        <v>5483</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>誠美材</t>
+          <t>中美晶</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>654.6452384080194</v>
+        <v>663.7168291409964</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>23.95</v>
+        <v>213.5</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,49 +3308,49 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>59.48442535256803</v>
+        <v>60.55907416121683</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>26.5034994712176</v>
+        <v>31.10196452451822</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.3855730370841804</v>
+        <v>0.3106851250175323</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M54" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.09992419299283251</v>
+        <v>2.478466658357904</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, invest_trust_buy_2d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>4908</v>
+        <v>4960</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>前鼎</t>
+          <t>誠美材</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>653.7951625943281</v>
+        <v>654.6452384080194</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>243</v>
+        <v>23.95</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>59.82274119936438</v>
+        <v>59.48442535256803</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>29.53550377010288</v>
+        <v>26.5034994712176</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.5675271399248706</v>
+        <v>0.3855730370841804</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.7151712078527233</v>
+        <v>0.09992419299283251</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6114</v>
+        <v>4908</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>久威</t>
+          <t>前鼎</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>645.6703505723137</v>
+        <v>653.7951625943281</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>24.85</v>
+        <v>243</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>53.0700414422202</v>
+        <v>59.82274119936438</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>14.73452530683979</v>
+        <v>29.53550377010288</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>4.287820650357013</v>
+        <v>0.5675271399248706</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.4974044485987643</v>
+        <v>0.7151712078527233</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>volume_break, breakout_20d, market_above_ma60, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>4956</v>
+        <v>6114</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>光鋐</t>
+          <t>久威</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>644.9424058999195</v>
+        <v>645.6703505723137</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>42.5</v>
+        <v>24.85</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,16 +3467,16 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>54.81819476715735</v>
+        <v>53.0700414422202</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>39.35281953366655</v>
+        <v>14.73452530683979</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.1890693428641503</v>
+        <v>4.287820650357013</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.4118607575555124</v>
+        <v>0.4974044485987643</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, breakout_20d, market_above_ma60, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>6005</v>
+        <v>4956</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>群益證</t>
+          <t>光鋐</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>644.5863469895137</v>
+        <v>644.9424058999195</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>32.75</v>
+        <v>42.5</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,16 +3520,16 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>55.3412403121324</v>
+        <v>54.81819476715735</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>12.36503781598968</v>
+        <v>39.35281953366655</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.9164527460567876</v>
+        <v>0.1890693428641503</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.09425326345158511</v>
+        <v>-0.4118607575555124</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>4961</v>
+        <v>6005</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>天鈺</t>
+          <t>群益證</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>644.5172716162623</v>
+        <v>644.5863469895137</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>174.5</v>
+        <v>32.75</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,49 +3573,49 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>46.14863984742773</v>
+        <v>55.3412403121324</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>21.44987062931387</v>
+        <v>12.36503781598968</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.5084745461122676</v>
+        <v>0.9164527460567876</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L59" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M59" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-1.170527277246571</v>
+        <v>0.09425326345158511</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, invest_trust_buy_2d, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>4545</v>
+        <v>4961</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>銘鈺</t>
+          <t>天鈺</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>631.7488702638526</v>
+        <v>644.5172716162623</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>37.9</v>
+        <v>174.5</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,49 +3626,49 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>64.21543580812184</v>
+        <v>46.14863984742773</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>38.3592927258088</v>
+        <v>21.44987062931387</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.8506210390889309</v>
+        <v>0.5084745461122676</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L60" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M60" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.2908168041301353</v>
+        <v>-1.170527277246571</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, invest_trust_buy_2d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>5493</v>
+        <v>4545</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>三聯</t>
+          <t>銘鈺</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>622.8949736605832</v>
+        <v>631.7488702638526</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>90.7</v>
+        <v>37.9</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>60.50680811202852</v>
+        <v>64.21543580812184</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>46.23467197317049</v>
+        <v>38.3592927258088</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.4296157859858127</v>
+        <v>0.8506210390889309</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.1503968914116487</v>
+        <v>0.2908168041301353</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3707,21 +3707,21 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>5521</v>
+        <v>5493</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>工信</t>
+          <t>三聯</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>622.0154782887736</v>
+        <v>622.8949736605832</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>11.05</v>
+        <v>90.7</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,16 +3732,16 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>66.23540953352483</v>
+        <v>60.50680811202852</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>21.52629223601599</v>
+        <v>46.23467197317049</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>1.147601583934789</v>
+        <v>0.4296157859858127</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.0534537295243965</v>
+        <v>-0.1503968914116487</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6108</v>
+        <v>5521</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>競國</t>
+          <t>工信</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>620.2698466004118</v>
+        <v>622.0154782887736</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>25.95</v>
+        <v>11.05</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,13 +3785,13 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>65.33864638149132</v>
+        <v>66.23540953352483</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>35.97234799595292</v>
+        <v>21.52629223601599</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>1.025395713392592</v>
+        <v>1.147601583934789</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>1</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.0796635274351172</v>
+        <v>0.0534537295243965</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>5452</v>
+        <v>6108</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>佶優</t>
+          <t>競國</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>620.212410937045</v>
+        <v>620.2698466004118</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>29.65</v>
+        <v>25.95</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>58.26078109939814</v>
+        <v>65.33864638149132</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>21.85614974818217</v>
+        <v>35.97234799595292</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.7798721634406347</v>
+        <v>1.025395713392592</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>1</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.351348609222323</v>
+        <v>0.0796635274351172</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>5353</v>
+        <v>5452</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>台林</t>
+          <t>佶優</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>619.2440680571153</v>
+        <v>620.212410937045</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>28.95</v>
+        <v>29.65</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,16 +3891,16 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>61.27187712034146</v>
+        <v>58.26078109939814</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>32.9067450920222</v>
+        <v>21.85614974818217</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.5624777500889997</v>
+        <v>0.7798721634406347</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.1038193999024781</v>
+        <v>0.351348609222323</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>6154</v>
+        <v>5353</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>順發</t>
+          <t>台林</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>615.3206360615621</v>
+        <v>619.2440680571153</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>14.25</v>
+        <v>28.95</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,16 +3944,16 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>60.5355941293179</v>
+        <v>61.27187712034146</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>34.53594234502944</v>
+        <v>32.9067450920222</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.7899432908249633</v>
+        <v>0.5624777500889997</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.0019400002804079</v>
+        <v>0.1038193999024781</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>4923</v>
+        <v>6154</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>力士</t>
+          <t>順發</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>608.2418861883608</v>
+        <v>615.3206360615621</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>57.2</v>
+        <v>14.25</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,16 +3997,16 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>46.58504387108941</v>
+        <v>60.5355941293179</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>28.93756565660965</v>
+        <v>34.53594234502944</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.4460942227803637</v>
+        <v>0.7899432908249633</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.6002477923441649</v>
+        <v>0.0019400002804079</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>5608</v>
+        <v>4923</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>四維航</t>
+          <t>力士</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>605.217076787305</v>
+        <v>608.2418861883608</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>17</v>
+        <v>57.2</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,16 +4050,16 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>54.68369152022238</v>
+        <v>46.58504387108941</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>28.78334121094643</v>
+        <v>28.93756565660965</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>1.892130838104808</v>
+        <v>0.4460942227803637</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.0847780175409725</v>
+        <v>-0.6002477923441649</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, williams_r_recovery, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>5203</v>
+        <v>5608</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>訊連</t>
+          <t>四維航</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>597.1663509199324</v>
+        <v>605.217076787305</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>60.5</v>
+        <v>17</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>57.76408559350125</v>
+        <v>54.68369152022238</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>29.54310581443301</v>
+        <v>28.78334121094643</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.6129467659701738</v>
+        <v>1.892130838104808</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>1</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.430588324530802</v>
+        <v>-0.0847780175409725</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, williams_r_recovery, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>5515</v>
+        <v>5203</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>建國</t>
+          <t>訊連</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>595.107294035933</v>
+        <v>597.1663509199324</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>52.4</v>
+        <v>60.5</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,16 +4156,16 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>58.56380392016354</v>
+        <v>57.76408559350125</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>17.01645841251321</v>
+        <v>29.54310581443301</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>1.043160638901905</v>
+        <v>0.6129467659701738</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.0621091111329525</v>
+        <v>0.430588324530802</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>5464</v>
+        <v>5515</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>霖宏</t>
+          <t>建國</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>594.9009807196139</v>
+        <v>595.107294035933</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>86.59999999999999</v>
+        <v>52.4</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>49.81264431604128</v>
+        <v>58.56380392016354</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>48.0617692056537</v>
+        <v>17.01645841251321</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>1.28085288778989</v>
+        <v>1.043160638901905</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.6520861879892275</v>
+        <v>0.0621091111329525</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>4919</v>
+        <v>5464</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>新唐</t>
+          <t>霖宏</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>588.3137989583253</v>
+        <v>594.9009807196139</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>154</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>63.11939133518563</v>
+        <v>49.81264431604128</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>35.5783891037951</v>
+        <v>48.0617692056537</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.9396334308381884</v>
+        <v>1.28085288778989</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>2.519023532190461</v>
+        <v>-0.6520861879892275</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>5234</v>
+        <v>4919</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>達興材料</t>
+          <t>新唐</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>588.2563970313257</v>
+        <v>588.3137989583253</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>319.5</v>
+        <v>154</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>54.9658391124597</v>
+        <v>63.11939133518563</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>31.83728211564337</v>
+        <v>35.5783891037951</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>1.342180444584764</v>
+        <v>0.9396334308381884</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>4.237317631599305</v>
+        <v>2.519023532190461</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>5220</v>
+        <v>5234</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>萬達光電</t>
+          <t>達興材料</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>586.7996133491008</v>
+        <v>588.2563970313257</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>22.25</v>
+        <v>319.5</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>60.94541953898941</v>
+        <v>54.9658391124597</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>30.23599777824747</v>
+        <v>31.83728211564337</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.3552811338660491</v>
+        <v>1.342180444584764</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,48 +4386,48 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.1134146054370546</v>
+        <v>4.237317631599305</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>4987</v>
+        <v>5220</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>科誠</t>
+          <t>萬達光電</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>584.8800228060522</v>
+        <v>586.7996133491008</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>81.59999999999999</v>
+        <v>22.25</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G75" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>55.06253860983202</v>
+        <v>60.94541953898941</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>23.90866292624774</v>
+        <v>30.23599777824747</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.750864911342356</v>
+        <v>0.3552811338660491</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,51 +4439,51 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.0408826678783921</v>
+        <v>0.1134146054370546</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6112</v>
+        <v>4987</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>邁達特</t>
+          <t>科誠</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>583.3958863754033</v>
+        <v>584.8800228060522</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>46.45</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="G76" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>49.78338712733051</v>
+        <v>55.06253860983202</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>29.83351204811389</v>
+        <v>23.90866292624774</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.2839752484377974</v>
+        <v>0.750864911342356</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.4480787889693133</v>
+        <v>-0.0408826678783921</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, dealer_buy_3d, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>5344</v>
+        <v>6112</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>立衛</t>
+          <t>邁達特</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>582.2183336817332</v>
+        <v>583.3958863754033</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>14.05</v>
+        <v>46.45</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,16 +4527,16 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>56.2204324137926</v>
+        <v>49.78338712733051</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>30.63727568572968</v>
+        <v>29.83351204811389</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.4808646108543982</v>
+        <v>0.2839752484377974</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.1080632795408715</v>
+        <v>-0.4480787889693133</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, dealer_buy_3d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6155</v>
+        <v>5344</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>鈞寶</t>
+          <t>立衛</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>582.0213177789625</v>
+        <v>582.2183336817332</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>70.2</v>
+        <v>14.05</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,49 +4580,49 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>64.00444112745816</v>
+        <v>56.2204324137926</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>27.20400987485574</v>
+        <v>30.63727568572968</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.7306239003907778</v>
+        <v>0.4808646108543982</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M78" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>1.142396850838091</v>
+        <v>0.1080632795408715</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>5465</v>
+        <v>6155</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>富驊</t>
+          <t>鈞寶</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>580.6136028992819</v>
+        <v>582.0213177789625</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>33.6</v>
+        <v>70.2</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,49 +4633,49 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>70.79064818882163</v>
+        <v>64.00444112745816</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>42.76143294262802</v>
+        <v>27.20400987485574</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.7062334963730383</v>
+        <v>0.7306239003907778</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L79" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M79" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.0881555487953154</v>
+        <v>1.142396850838091</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>5228</v>
+        <v>5465</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>鈺鎧</t>
+          <t>富驊</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>574.2585742461667</v>
+        <v>580.6136028992819</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>59.6</v>
+        <v>33.6</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,13 +4686,13 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>78.41026952974192</v>
+        <v>70.79064818882163</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>29.68932659357424</v>
+        <v>42.76143294262802</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>5.852141042021944</v>
+        <v>0.7062334963730383</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>2.339268306821928</v>
+        <v>0.0881555487953154</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6134</v>
+        <v>5228</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>萬旭</t>
+          <t>鈺鎧</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>573.0759903996541</v>
+        <v>574.2585742461667</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>27.9</v>
+        <v>59.6</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,16 +4739,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>40.13812732806851</v>
+        <v>78.41026952974192</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>22.42414105478816</v>
+        <v>29.68932659357424</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.7130375256029251</v>
+        <v>5.852141042021944</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.1452697340841046</v>
+        <v>2.339268306821928</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>4807</v>
+        <v>6134</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>日成-KY</t>
+          <t>萬旭</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>571.2932504433859</v>
+        <v>573.0759903996541</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>33.25</v>
+        <v>27.9</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,16 +4792,16 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>61.5741522257397</v>
+        <v>40.13812732806851</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>30.32955891710772</v>
+        <v>22.42414105478816</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>1.069146331681389</v>
+        <v>0.7130375256029251</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.5320790333747728</v>
+        <v>-0.1452697340841046</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>5292</v>
+        <v>4807</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>華懋</t>
+          <t>日成-KY</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>569.0401435797967</v>
+        <v>571.2932504433859</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>243.5</v>
+        <v>33.25</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,16 +4845,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>67.42915489680026</v>
+        <v>61.5741522257397</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>32.35848777140647</v>
+        <v>30.32955891710772</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.6441049896818133</v>
+        <v>1.069146331681389</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>1.523786696622086</v>
+        <v>0.5320790333747728</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>4935</v>
+        <v>5292</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>茂林-KY</t>
+          <t>華懋</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>566.2655419919755</v>
+        <v>569.0401435797967</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>34.4</v>
+        <v>243.5</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,16 +4898,16 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>57.24769157328625</v>
+        <v>67.42915489680026</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>23.94365451625797</v>
+        <v>32.35848777140647</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.5789421501309648</v>
+        <v>0.6441049896818133</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.1952647015061191</v>
+        <v>1.523786696622086</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>4577</v>
+        <v>4935</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>達航科技</t>
+          <t>茂林-KY</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>545.7493818363199</v>
+        <v>566.2655419919755</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>90.09999999999999</v>
+        <v>34.4</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,16 +4951,16 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>56.86653957053161</v>
+        <v>57.24769157328625</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>32.24446055486187</v>
+        <v>23.94365451625797</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.4584572683301938</v>
+        <v>0.5789421501309648</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.0856075902445308</v>
+        <v>0.1952647015061191</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>5425</v>
+        <v>4577</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>台半</t>
+          <t>達航科技</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>545.0846281885548</v>
+        <v>545.7493818363199</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>100.5</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,16 +5004,16 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>56.93522810649883</v>
+        <v>56.86653957053161</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>25.57354807857544</v>
+        <v>32.24446055486187</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.3261091928158386</v>
+        <v>0.4584572683301938</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.6131674081887546</v>
+        <v>0.0856075902445308</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>4729</v>
+        <v>5425</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>熒茂</t>
+          <t>台半</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>541.2208465832859</v>
+        <v>545.0846281885548</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>19.75</v>
+        <v>100.5</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,16 +5057,16 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>56.86803887307256</v>
+        <v>56.93522810649883</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>26.43764874380561</v>
+        <v>25.57354807857544</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.4994403479219657</v>
+        <v>0.3261091928158386</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.07745861048419771</v>
+        <v>0.6131674081887546</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>5536</v>
+        <v>4729</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>聖暉*</t>
+          <t>熒茂</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>537.1542701194419</v>
+        <v>541.2208465832859</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>931</v>
+        <v>19.75</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,49 +5110,49 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>50.55313518586189</v>
+        <v>56.86803887307256</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>26.34158690844838</v>
+        <v>26.43764874380561</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>1.986706030333102</v>
+        <v>0.4994403479219657</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L88" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="M88" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>13.47100459860625</v>
+        <v>0.07745861048419771</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, invest_trust_buy_2d, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>4736</v>
+        <v>5536</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>泰博</t>
+          <t>聖暉*</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>536.8573296440838</v>
+        <v>537.1542701194419</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>133.5</v>
+        <v>931</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,49 +5163,49 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>57.47894563634589</v>
+        <v>50.55313518586189</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>17.19209443702598</v>
+        <v>26.34158690844838</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>1.408186737991385</v>
+        <v>1.986706030333102</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L89" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="M89" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.454433313862074</v>
+        <v>13.47100459860625</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, invest_trust_buy_2d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>5289</v>
+        <v>4736</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>宜鼎</t>
+          <t>泰博</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>535.6843045212275</v>
+        <v>536.8573296440838</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>1260</v>
+        <v>133.5</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,49 +5216,49 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>38.49579712621616</v>
+        <v>57.47894563634589</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>16.00113180418879</v>
+        <v>17.19209443702598</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>1.066508673929769</v>
+        <v>1.408186737991385</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L90" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M90" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>1.963991164919513</v>
+        <v>0.454433313862074</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, invest_trust_buy_2d, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>4526</v>
+        <v>5289</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>東台</t>
+          <t>宜鼎</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>527.8349119990253</v>
+        <v>535.6843045212275</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>32.6</v>
+        <v>1260</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,49 +5269,49 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>52.11211548630438</v>
+        <v>38.49579712621616</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>27.02539418194234</v>
+        <v>16.00113180418879</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.4140042089518226</v>
+        <v>1.066508673929769</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L91" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M91" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>0.0467327506067659</v>
+        <v>1.963991164919513</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, invest_trust_buy_2d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6113</v>
+        <v>4526</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>亞矽</t>
+          <t>東台</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>525.3146747221708</v>
+        <v>527.8349119990253</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>23.8</v>
+        <v>32.6</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,16 +5322,16 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>56.56423108033362</v>
+        <v>52.11211548630438</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>22.34165652710811</v>
+        <v>27.02539418194234</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.7802263270330195</v>
+        <v>0.4140042089518226</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L92" s="2" t="n">
         <v>0</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.1495502890080536</v>
+        <v>0.0467327506067659</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>4739</v>
+        <v>6113</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>康普</t>
+          <t>亞矽</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>523.8487465086052</v>
+        <v>525.3146747221708</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>88.7</v>
+        <v>23.8</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>59.82964527285116</v>
+        <v>56.56423108033362</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>22.21057430709613</v>
+        <v>22.34165652710811</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.8982398409582816</v>
+        <v>0.7802263270330195</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>1</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.8925454898344864</v>
+        <v>0.1495502890080536</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>4905</v>
+        <v>4739</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>台聯電</t>
+          <t>康普</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>520.2204144311797</v>
+        <v>523.8487465086052</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>88.90000000000001</v>
+        <v>88.7</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,13 +5428,13 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>56.68235080252865</v>
+        <v>59.82964527285116</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>16.02982050437717</v>
+        <v>22.21057430709613</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.6220414431179692</v>
+        <v>0.8982398409582816</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>1</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>1.021721199938096</v>
+        <v>0.8925454898344864</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>4924</v>
+        <v>4905</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>欣厚-KY</t>
+          <t>台聯電</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>518.3529620957129</v>
+        <v>520.2204144311797</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>16.75</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,16 +5481,16 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>60.38702056765914</v>
+        <v>56.68235080252865</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>31.278267782731</v>
+        <v>16.02982050437717</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.9220434012848716</v>
+        <v>0.6220414431179692</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.0790424927438842</v>
+        <v>1.021721199938096</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>4915</v>
+        <v>4924</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>致伸</t>
+          <t>欣厚-KY</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>510.2091949630552</v>
+        <v>518.3529620957129</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>63.4</v>
+        <v>16.75</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>50.39436042620808</v>
+        <v>60.38702056765914</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>27.40277801768876</v>
+        <v>31.278267782731</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.4299852187908243</v>
+        <v>0.9220434012848716</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.1818347792595935</v>
+        <v>-0.0790424927438842</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>4766</v>
+        <v>4915</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>南寶</t>
+          <t>致伸</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>504.411319819162</v>
+        <v>510.2091949630552</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>355.5</v>
+        <v>63.4</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,16 +5587,16 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>59.98039692462093</v>
+        <v>50.39436042620808</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>18.89329806482605</v>
+        <v>27.40277801768876</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.9735417408632072</v>
+        <v>0.4299852187908243</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>1.488436198288973</v>
+        <v>-0.1818347792595935</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>4991</v>
+        <v>4766</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>環宇-KY</t>
+          <t>南寶</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>503.2182996263965</v>
+        <v>504.411319819162</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>510</v>
+        <v>355.5</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,49 +5640,49 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>54.73959611976854</v>
+        <v>59.98039692462093</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>12.67563901372659</v>
+        <v>18.89329806482605</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>1.321218644770261</v>
+        <v>0.9735417408632072</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L98" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M98" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>4.557315320607682</v>
+        <v>1.488436198288973</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>4576</v>
+        <v>4991</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>大銀微系統</t>
+          <t>環宇-KY</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>499.3374967983433</v>
+        <v>503.2182996263965</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>233.5</v>
+        <v>510</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,49 +5693,49 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>52.37523486578827</v>
+        <v>54.73959611976854</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>16.51179348934591</v>
+        <v>12.67563901372659</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>1.165103568337306</v>
+        <v>1.321218644770261</v>
       </c>
       <c r="K99" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L99" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L99" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M99" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-1.09031670216579</v>
+        <v>4.557315320607682</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>5351</v>
+        <v>4576</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>鈺創</t>
+          <t>大銀微系統</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>498.0479212288383</v>
+        <v>499.3374967983433</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>114</v>
+        <v>233.5</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,13 +5746,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>53.33673661542694</v>
+        <v>52.37523486578827</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>14.29227870359377</v>
+        <v>16.51179348934591</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.5815541195145947</v>
+        <v>1.165103568337306</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>1</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.4937770147566389</v>
+        <v>-1.09031670216579</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>6103</v>
+        <v>5351</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>合邦</t>
+          <t>鈺創</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>497.5411557977713</v>
+        <v>498.0479212288383</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>38.6</v>
+        <v>114</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,16 +5799,16 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>54.01386918700866</v>
+        <v>53.33673661542694</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>6.809419748977756</v>
+        <v>14.29227870359377</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.5052284318681584</v>
+        <v>0.5815541195145947</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.2270444506609004</v>
+        <v>0.4937770147566389</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>4749</v>
+        <v>6103</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>新應材</t>
+          <t>合邦</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>496.2964873939864</v>
+        <v>497.5411557977713</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>737</v>
+        <v>38.6</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,49 +5852,49 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>43.53141973553147</v>
+        <v>54.01386918700866</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>17.83487571476568</v>
+        <v>6.809419748977756</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.9502823557022492</v>
+        <v>0.5052284318681584</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L102" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M102" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>2.73615477161345</v>
+        <v>-0.2270444506609004</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, invest_trust_buy_2d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>5356</v>
+        <v>4749</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>協益</t>
+          <t>新應材</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>479.5378503409824</v>
+        <v>496.2964873939864</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>25.9</v>
+        <v>737</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,49 +5905,49 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>51.86977789934928</v>
+        <v>43.53141973553147</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>24.35999469359081</v>
+        <v>17.83487571476568</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>3.527687180849545</v>
+        <v>0.9502823557022492</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L103" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M103" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.006195975862899</v>
+        <v>2.73615477161345</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, invest_trust_buy_2d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6127</v>
+        <v>5356</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>九豪</t>
+          <t>協益</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>479.2275388421416</v>
+        <v>479.5378503409824</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>64</v>
+        <v>25.9</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>74.00011368791687</v>
+        <v>51.86977789934928</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>26.38051128267922</v>
+        <v>24.35999469359081</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>4.677731675619241</v>
+        <v>3.527687180849545</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,11 +5976,11 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>1.625777226958198</v>
+        <v>-0.006195975862899</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
@@ -7099,21 +7099,21 @@
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
-        <v>6120</v>
+        <v>6126</v>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>達運</t>
+          <t>信音</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>423.816327374783</v>
+        <v>429.0857046278272</v>
       </c>
       <c r="E126" s="2" t="n">
-        <v>13.45</v>
+        <v>30.85</v>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
@@ -7124,49 +7124,49 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>51.90793970070203</v>
+        <v>49.4947653520305</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>36.53475207312602</v>
+        <v>34.55141294149456</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>0.4492421789382883</v>
+        <v>1.275545021697343</v>
       </c>
       <c r="K126" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L126" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M126" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>0.0509933151758916</v>
+        <v>0.108412450297581</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
-        <v>4771</v>
+        <v>6120</v>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>望隼</t>
+          <t>達運</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
         <v/>
       </c>
       <c r="D127" s="2" t="n">
-        <v>422.3480957550432</v>
+        <v>423.816327374783</v>
       </c>
       <c r="E127" s="2" t="n">
-        <v>206</v>
+        <v>13.45</v>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
@@ -7177,49 +7177,49 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>46.93887367852542</v>
+        <v>51.90793970070203</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>15.08514286642427</v>
+        <v>36.53475207312602</v>
       </c>
       <c r="J127" s="2" t="n">
-        <v>0.529502470729812</v>
+        <v>0.4492421789382883</v>
       </c>
       <c r="K127" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L127" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M127" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-1.495165859835996</v>
+        <v>0.0509933151758916</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
-        <v>4971</v>
+        <v>4771</v>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>IET-KY</t>
+          <t>望隼</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
         <v/>
       </c>
       <c r="D128" s="2" t="n">
-        <v>420.5432797976616</v>
+        <v>422.3480957550432</v>
       </c>
       <c r="E128" s="2" t="n">
-        <v>590</v>
+        <v>206</v>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
@@ -7230,13 +7230,13 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>54.6906958426387</v>
+        <v>46.93887367852542</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>14.9037832729082</v>
+        <v>15.08514286642427</v>
       </c>
       <c r="J128" s="2" t="n">
-        <v>0.5787322611067528</v>
+        <v>0.529502470729812</v>
       </c>
       <c r="K128" s="2" t="n">
         <v>0</v>
@@ -7248,31 +7248,31 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>2.138585484350686</v>
+        <v>-1.495165859835996</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
-        <v>4555</v>
+        <v>4971</v>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>氣立</t>
+          <t>IET-KY</t>
         </is>
       </c>
       <c r="C129" s="2" t="n">
         <v/>
       </c>
       <c r="D129" s="2" t="n">
-        <v>415.9751154992992</v>
+        <v>420.5432797976616</v>
       </c>
       <c r="E129" s="2" t="n">
-        <v>43.2</v>
+        <v>590</v>
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
@@ -7283,16 +7283,16 @@
         <v>0</v>
       </c>
       <c r="H129" s="2" t="n">
-        <v>50.68397748770373</v>
+        <v>54.6906958426387</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>12.49823015659547</v>
+        <v>14.9037832729082</v>
       </c>
       <c r="J129" s="2" t="n">
-        <v>1.126157381324306</v>
+        <v>0.5787322611067528</v>
       </c>
       <c r="K129" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L129" s="2" t="n">
         <v>0</v>
@@ -7301,31 +7301,31 @@
         <v>-1</v>
       </c>
       <c r="N129" s="2" t="n">
-        <v>0.2113512353941353</v>
+        <v>2.138585484350686</v>
       </c>
       <c r="O129" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
-        <v>4581</v>
+        <v>4555</v>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>光隆精密-KY</t>
+          <t>氣立</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
         <v/>
       </c>
       <c r="D130" s="2" t="n">
-        <v>413.5993544696796</v>
+        <v>415.9751154992992</v>
       </c>
       <c r="E130" s="2" t="n">
-        <v>48.2</v>
+        <v>43.2</v>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
@@ -7336,16 +7336,16 @@
         <v>0</v>
       </c>
       <c r="H130" s="2" t="n">
-        <v>51.84606279610517</v>
+        <v>50.68397748770373</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>9.886028082265479</v>
+        <v>12.49823015659547</v>
       </c>
       <c r="J130" s="2" t="n">
-        <v>0.821747021226229</v>
+        <v>1.126157381324306</v>
       </c>
       <c r="K130" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L130" s="2" t="n">
         <v>0</v>
@@ -7354,31 +7354,31 @@
         <v>-1</v>
       </c>
       <c r="N130" s="2" t="n">
-        <v>-1.657576563905997</v>
+        <v>0.2113512353941353</v>
       </c>
       <c r="O130" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, williams_r_recovery, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n">
-        <v>5299</v>
+        <v>4581</v>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>杰力</t>
+          <t>光隆精密-KY</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
         <v/>
       </c>
       <c r="D131" s="2" t="n">
-        <v>413.5292212002606</v>
+        <v>413.5993544696796</v>
       </c>
       <c r="E131" s="2" t="n">
-        <v>96.59999999999999</v>
+        <v>48.2</v>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
@@ -7389,16 +7389,16 @@
         <v>0</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>44.25569423831968</v>
+        <v>51.84606279610517</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>20.81190761816711</v>
+        <v>9.886028082265479</v>
       </c>
       <c r="J131" s="2" t="n">
-        <v>0.6867825444288495</v>
+        <v>0.821747021226229</v>
       </c>
       <c r="K131" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L131" s="2" t="n">
         <v>0</v>
@@ -7407,31 +7407,31 @@
         <v>-1</v>
       </c>
       <c r="N131" s="2" t="n">
-        <v>-0.0544981795435998</v>
+        <v>-1.657576563905997</v>
       </c>
       <c r="O131" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, williams_r_recovery, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n">
-        <v>5272</v>
+        <v>5299</v>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>笙科</t>
+          <t>杰力</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
         <v/>
       </c>
       <c r="D132" s="2" t="n">
-        <v>411.2302743851258</v>
+        <v>413.5292212002606</v>
       </c>
       <c r="E132" s="2" t="n">
-        <v>17.6</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
@@ -7442,13 +7442,13 @@
         <v>0</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>53.97822307826279</v>
+        <v>44.25569423831968</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>23.82570732741605</v>
+        <v>20.81190761816711</v>
       </c>
       <c r="J132" s="2" t="n">
-        <v>0.4586528574437245</v>
+        <v>0.6867825444288495</v>
       </c>
       <c r="K132" s="2" t="n">
         <v>0</v>
@@ -7460,31 +7460,31 @@
         <v>-1</v>
       </c>
       <c r="N132" s="2" t="n">
-        <v>0.06610704752952069</v>
+        <v>-0.0544981795435998</v>
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n">
-        <v>5706</v>
+        <v>5272</v>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>鳳凰</t>
+          <t>笙科</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
         <v/>
       </c>
       <c r="D133" s="2" t="n">
-        <v>409.7906812927858</v>
+        <v>411.2302743851258</v>
       </c>
       <c r="E133" s="2" t="n">
-        <v>44.35</v>
+        <v>17.6</v>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
@@ -7495,16 +7495,16 @@
         <v>0</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>48.85743101581013</v>
+        <v>53.97822307826279</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>14.93194110901488</v>
+        <v>23.82570732741605</v>
       </c>
       <c r="J133" s="2" t="n">
-        <v>1.278905514455314</v>
+        <v>0.4586528574437245</v>
       </c>
       <c r="K133" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L133" s="2" t="n">
         <v>0</v>
@@ -7513,31 +7513,31 @@
         <v>-1</v>
       </c>
       <c r="N133" s="2" t="n">
-        <v>0.0847410215913055</v>
+        <v>0.06610704752952069</v>
       </c>
       <c r="O133" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, kd_golden_cross, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n">
-        <v>6117</v>
+        <v>5706</v>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>迎廣</t>
+          <t>鳳凰</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
         <v/>
       </c>
       <c r="D134" s="2" t="n">
-        <v>409.1742840692721</v>
+        <v>409.7906812927858</v>
       </c>
       <c r="E134" s="2" t="n">
-        <v>64.7</v>
+        <v>44.35</v>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
@@ -7548,16 +7548,16 @@
         <v>0</v>
       </c>
       <c r="H134" s="2" t="n">
-        <v>54.60336661583372</v>
+        <v>48.85743101581013</v>
       </c>
       <c r="I134" s="2" t="n">
-        <v>26.93648161518508</v>
+        <v>14.93194110901488</v>
       </c>
       <c r="J134" s="2" t="n">
-        <v>0.8174284069272135</v>
+        <v>1.278905514455314</v>
       </c>
       <c r="K134" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L134" s="2" t="n">
         <v>0</v>
@@ -7566,31 +7566,31 @@
         <v>-1</v>
       </c>
       <c r="N134" s="2" t="n">
-        <v>0.6245815537372974</v>
+        <v>0.0847410215913055</v>
       </c>
       <c r="O134" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n">
-        <v>5251</v>
+        <v>6117</v>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>天鉞電</t>
+          <t>迎廣</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
         <v/>
       </c>
       <c r="D135" s="2" t="n">
-        <v>404.1421569746581</v>
+        <v>409.1742840692721</v>
       </c>
       <c r="E135" s="2" t="n">
-        <v>30</v>
+        <v>64.7</v>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
@@ -7601,13 +7601,13 @@
         <v>0</v>
       </c>
       <c r="H135" s="2" t="n">
-        <v>54.72683454594053</v>
+        <v>54.60336661583372</v>
       </c>
       <c r="I135" s="2" t="n">
-        <v>38.5332490936626</v>
+        <v>26.93648161518508</v>
       </c>
       <c r="J135" s="2" t="n">
-        <v>0.2822027279312083</v>
+        <v>0.8174284069272135</v>
       </c>
       <c r="K135" s="2" t="n">
         <v>0</v>
@@ -7619,31 +7619,31 @@
         <v>-1</v>
       </c>
       <c r="N135" s="2" t="n">
-        <v>-0.0947528175697578</v>
+        <v>0.6245815537372974</v>
       </c>
       <c r="O135" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
-        <v>4562</v>
+        <v>5251</v>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>穎漢</t>
+          <t>天鉞電</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
         <v/>
       </c>
       <c r="D136" s="2" t="n">
-        <v>403.4686852813243</v>
+        <v>404.1421569746581</v>
       </c>
       <c r="E136" s="2" t="n">
-        <v>30.7</v>
+        <v>30</v>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
@@ -7654,16 +7654,16 @@
         <v>0</v>
       </c>
       <c r="H136" s="2" t="n">
-        <v>52.43750410585558</v>
+        <v>54.72683454594053</v>
       </c>
       <c r="I136" s="2" t="n">
-        <v>15.80689830062943</v>
+        <v>38.5332490936626</v>
       </c>
       <c r="J136" s="2" t="n">
-        <v>0.883304730981504</v>
+        <v>0.2822027279312083</v>
       </c>
       <c r="K136" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L136" s="2" t="n">
         <v>0</v>
@@ -7672,31 +7672,31 @@
         <v>-1</v>
       </c>
       <c r="N136" s="2" t="n">
-        <v>0.0789297761023207</v>
+        <v>-0.0947528175697578</v>
       </c>
       <c r="O136" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, kd_golden_cross, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n">
-        <v>4763</v>
+        <v>4562</v>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>材料*-KY</t>
+          <t>穎漢</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
         <v/>
       </c>
       <c r="D137" s="2" t="n">
-        <v>393.6195766705927</v>
+        <v>403.4686852813243</v>
       </c>
       <c r="E137" s="2" t="n">
-        <v>46.85</v>
+        <v>30.7</v>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
@@ -7707,49 +7707,49 @@
         <v>0</v>
       </c>
       <c r="H137" s="2" t="n">
-        <v>47.11241320467021</v>
+        <v>52.43750410585558</v>
       </c>
       <c r="I137" s="2" t="n">
-        <v>15.35694493581871</v>
+        <v>15.80689830062943</v>
       </c>
       <c r="J137" s="2" t="n">
-        <v>0.4202933352994767</v>
+        <v>0.883304730981504</v>
       </c>
       <c r="K137" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L137" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M137" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N137" s="2" t="n">
-        <v>-0.0783998109085669</v>
+        <v>0.0789297761023207</v>
       </c>
       <c r="O137" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, invest_trust_buy_2d</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n">
-        <v>6139</v>
+        <v>4763</v>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>亞翔</t>
+          <t>材料*-KY</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
         <v/>
       </c>
       <c r="D138" s="2" t="n">
-        <v>393.3622295859685</v>
+        <v>393.6195766705927</v>
       </c>
       <c r="E138" s="2" t="n">
-        <v>750</v>
+        <v>46.85</v>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
@@ -7760,49 +7760,49 @@
         <v>0</v>
       </c>
       <c r="H138" s="2" t="n">
-        <v>48.47599604688763</v>
+        <v>47.11241320467021</v>
       </c>
       <c r="I138" s="2" t="n">
-        <v>16.48324879417975</v>
+        <v>15.35694493581871</v>
       </c>
       <c r="J138" s="2" t="n">
-        <v>1.152307236251471</v>
+        <v>0.4202933352994767</v>
       </c>
       <c r="K138" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L138" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M138" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N138" s="2" t="n">
-        <v>5.352287647578811</v>
+        <v>-0.0783998109085669</v>
       </c>
       <c r="O138" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, invest_trust_buy_2d</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n">
-        <v>5328</v>
+        <v>6139</v>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>華容</t>
+          <t>亞翔</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
         <v/>
       </c>
       <c r="D139" s="2" t="n">
-        <v>392.3888001140759</v>
+        <v>393.3622295859685</v>
       </c>
       <c r="E139" s="2" t="n">
-        <v>57.6</v>
+        <v>750</v>
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
@@ -7813,25 +7813,25 @@
         <v>0</v>
       </c>
       <c r="H139" s="2" t="n">
-        <v>51.71958048927354</v>
+        <v>48.47599604688763</v>
       </c>
       <c r="I139" s="2" t="n">
-        <v>19.75493667108496</v>
+        <v>16.48324879417975</v>
       </c>
       <c r="J139" s="2" t="n">
-        <v>0.4554184058459453</v>
+        <v>1.152307236251471</v>
       </c>
       <c r="K139" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L139" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M139" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N139" s="2" t="n">
-        <v>0.8082118821268409</v>
+        <v>5.352287647578811</v>
       </c>
       <c r="O139" s="2" t="inlineStr">
         <is>
@@ -7841,21 +7841,21 @@
     </row>
     <row r="140">
       <c r="A140" s="2" t="n">
-        <v>6126</v>
+        <v>5328</v>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>信音</t>
+          <t>華容</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
         <v/>
       </c>
       <c r="D140" s="2" t="n">
-        <v>389.0857046278282</v>
+        <v>392.3888001140759</v>
       </c>
       <c r="E140" s="2" t="n">
-        <v>30.85</v>
+        <v>57.6</v>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
@@ -7866,13 +7866,13 @@
         <v>0</v>
       </c>
       <c r="H140" s="2" t="n">
-        <v>49.49476538201494</v>
+        <v>51.71958048927354</v>
       </c>
       <c r="I140" s="2" t="n">
-        <v>34.55141291876783</v>
+        <v>19.75493667108496</v>
       </c>
       <c r="J140" s="2" t="n">
-        <v>1.275545021697343</v>
+        <v>0.4554184058459453</v>
       </c>
       <c r="K140" s="2" t="n">
         <v>0</v>
@@ -7884,11 +7884,11 @@
         <v>-1</v>
       </c>
       <c r="N140" s="2" t="n">
-        <v>0.1084124503456488</v>
+        <v>0.8082118821268409</v>
       </c>
       <c r="O140" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -10092,10 +10092,10 @@
         <v>0</v>
       </c>
       <c r="H182" s="2" t="n">
-        <v>49.79827510888917</v>
+        <v>49.79827523723347</v>
       </c>
       <c r="I182" s="2" t="n">
-        <v>17.01701478825803</v>
+        <v>17.01701484026341</v>
       </c>
       <c r="J182" s="2" t="n">
         <v>1.274024330381658</v>
@@ -10110,7 +10110,7 @@
         <v>-1</v>
       </c>
       <c r="N182" s="2" t="n">
-        <v>0.2145950048902838</v>
+        <v>0.2145950038567886</v>
       </c>
       <c r="O182" s="2" t="inlineStr">
         <is>
@@ -11099,10 +11099,10 @@
         <v>0</v>
       </c>
       <c r="H201" s="2" t="n">
-        <v>43.9586939433886</v>
+        <v>43.95869352314547</v>
       </c>
       <c r="I201" s="2" t="n">
-        <v>21.5471296241776</v>
+        <v>21.54712953931656</v>
       </c>
       <c r="J201" s="2" t="n">
         <v>0.5836220315589363</v>
@@ -11117,7 +11117,7 @@
         <v>-1</v>
       </c>
       <c r="N201" s="2" t="n">
-        <v>-0.0423734948118643</v>
+        <v>-0.0423734947294825</v>
       </c>
       <c r="O201" s="2" t="inlineStr">
         <is>

</xml_diff>